<commit_message>
Update TS4_mapping.xlsx via Streamlit
</commit_message>
<xml_diff>
--- a/TS4_mapping.xlsx
+++ b/TS4_mapping.xlsx
@@ -573,8 +573,14 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+      <c r="E2" t="n">
+        <v>64265166440004</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
@@ -585,8 +591,16 @@
       </c>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>AOT</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>fiber_check-parse_cpo_data_collect_results-FAIL-MEASUREMENT;</t>
+        </is>
+      </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
@@ -617,8 +631,14 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
+      <c r="E3" t="n">
+        <v>64265166440005</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
@@ -629,8 +649,16 @@
       </c>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>AOT</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>cpld_revision-bmc_cpld_fu_interface_test-FAIL-MEASUREMENT;</t>
+        </is>
+      </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
@@ -661,8 +689,14 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+      <c r="E4" t="n">
+        <v>64265166440003</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
@@ -673,7 +707,11 @@
       </c>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>AOT</t>
+        </is>
+      </c>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
@@ -705,8 +743,14 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
+      <c r="E5" t="n">
+        <v>64265166440001</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
@@ -717,8 +761,16 @@
       </c>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>AOT</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>initial_setup-mft_revision-FAIL-MEASUREMENT;</t>
+        </is>
+      </c>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
@@ -749,8 +801,14 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
+      <c r="E6" t="n">
+        <v>64265166440002</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
@@ -761,8 +819,16 @@
       </c>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>AOT</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>cpld_revision-bmc_cpld_fu_interface_test-FAIL-MEASUREMENT;</t>
+        </is>
+      </c>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>

</xml_diff>